<commit_message>
Major changes to My account and addition of dynamic waits
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/DashboardData.xlsx
+++ b/src/test/resources/TEST_DATA/DashboardData.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="4"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="DashboardSavingsValidationData" sheetId="1" state="visible" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t>savingsAccountNumber</t>
   </si>
@@ -79,7 +79,10 @@
     <t>loanPeriod</t>
   </si>
   <si>
-    <t>300164007642</t>
+    <t>300164007643</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LKR -5,000.00</t>
   </si>
   <si>
     <t xml:space="preserve">LKR 5,000.00</t>
@@ -157,7 +160,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -166,6 +169,7 @@
     <xf fontId="2" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf fontId="0" fillId="0" borderId="0" numFmtId="49" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -792,17 +796,17 @@
       <c r="A2" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="4" t="s">
         <v>20</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -819,12 +823,12 @@
   <sheetData>
     <row r="1" ht="14.25">
       <c r="A1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="2" ht="14.25">
       <c r="A2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
   </sheetData>
@@ -846,24 +850,24 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Changes to execution plan and stabilization
</commit_message>
<xml_diff>
--- a/src/test/resources/TEST_DATA/DashboardData.xlsx
+++ b/src/test/resources/TEST_DATA/DashboardData.xlsx
@@ -82,10 +82,10 @@
     <t>300164007643</t>
   </si>
   <si>
+    <t xml:space="preserve">LKR 5,000.00</t>
+  </si>
+  <si>
     <t xml:space="preserve">LKR -5,000.00</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LKR 5,000.00</t>
   </si>
   <si>
     <t>12</t>
@@ -799,7 +799,7 @@
       <c r="B2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="4" t="s">
         <v>21</v>
       </c>
       <c r="D2" s="1" t="s">

</xml_diff>